<commit_message>
feat: update department hierarchy to 4-level structure
- KPTCL_Substation_Mapping.xlsx: rebuilt Master sheet as 4-level
  hierarchy (Zone → Circle → Division → Station Name) from SIS code
  circular; station names now voltage-prefixed (e.g. 220kV BIAL Begur)
- equipment_seed.xlsx: Departments sheet reduced to 4 columns
  (zone, circle, division, substation); circle/division values aligned
  to Master sheet; 4 mismatched station names corrected to match seeded
  department names (EDC, Kanakapura, Manyatha Tech Park, DHP)
- seed.py: seed_kptcl_departments now derives hierarchy levels
  dynamically from Excel columns instead of hardcoded 6-level list

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/equipment_seed.xlsx
+++ b/equipment_seed.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -39,8 +39,12 @@
       <name val="Arial"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -53,8 +57,13 @@
         <bgColor rgb="001F4E79"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E79"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -68,16 +77,36 @@
       <top style="thin"/>
       <bottom style="thin"/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00BFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -443,396 +472,276 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F12"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <dimension ref="A1:D12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="33" customWidth="1" min="2" max="2"/>
-    <col width="21" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
     <col width="30" customWidth="1" min="5" max="5"/>
     <col width="28" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="25" customHeight="1">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>zone</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>circle</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
         <is>
           <t>division</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>sub_division</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>section</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="D1" s="3" t="inlineStr">
         <is>
           <t>substation</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Bengaluru Zone</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Bengaluru Transmission Circle</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>RT North Division</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>RT North SD3 Devanahalli</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>BIAL Begur Section</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>Bangalore Zone</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>BRAZ</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>Begur</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
         <is>
           <t>220kV BIAL Begur</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>Bengaluru Zone</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>Bengaluru Transmission Circle</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>RT East Division</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>RT East SD4 Anekal</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>EDC Section</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>220kV EDC</t>
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Bangalore Zone</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>BMAZ South</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Hoody</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>Bengaluru Zone</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>Bengaluru Transmission Circle</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>RT East Division</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>RT East SD4 Anekal</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>Jigani Section</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Bangalore Zone</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Ramanagara</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Yerandanahally</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>220kV Jigani</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>Bengaluru Zone</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>Bengaluru Transmission Circle</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>RT South Division</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>RT South SD4 Kanakapura</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>Kanakapura Section</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>220kV Kanakapura</t>
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Bangalore Zone</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Ramanagara</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Kanakapura</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>220kV Kanakpura</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>Bengaluru Zone</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>Kolar Transmission Circle</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Kolar Division</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>Kolar SD1</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>Kolar Town Section</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Bangalore Zone</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>BRAZ</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Kolar</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
         <is>
           <t>220kV Kolar</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>Bengaluru Zone</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>Kolar Transmission Circle</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>Kolar Division</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>Malur SD</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>Malur Section</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Bangalore Zone</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>BRAZ</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Malur</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
         <is>
           <t>220kV Malur</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>Bengaluru Zone</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>Bengaluru Transmission Circle</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>RT North Division</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>RT North SD2 Hebbal</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>Manyatha Tech Park Section</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>220kV Manyatha Tech Park</t>
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Bangalore Zone</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>BMAZ North</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Hebbal</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>220kV Manyatha Tech Park GIS Station</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>Bengaluru Zone</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>Bengaluru Transmission Circle</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>RT South Division</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>RT South SD1 Rajajinagar</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>Rajajinagar Section</t>
-        </is>
-      </c>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Bangalore Zone</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>BMAZ North</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>NRS</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
         <is>
           <t>220kV NRS Rajajinagar</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>Bengaluru Zone</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>Bengaluru Transmission Circle</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>RT East Division</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>RT East SD1 Whitefield</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>Sarjapura Section</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Bangalore Zone</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Ramanagara</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Yerandanahally</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
         <is>
           <t>220kV Sarjapura</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>Bengaluru Zone</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>Bengaluru Transmission Circle</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>RT East Division</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>RT East SD1 Whitefield</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>DHP Section</t>
-        </is>
-      </c>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>400kV DHP</t>
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Bangalore Zone</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>BRAZ</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Devanahalli Hardware Park</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>400kV Devanahalli Hardware Park</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>Bengaluru Zone</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>Bengaluru Transmission Circle</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>RT East Division</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>RT East SD1 Whitefield</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>Hoody Section</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Bangalore Zone</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>BMAZ South</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>Hoody</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
         <is>
           <t>400kV Hoody</t>
         </is>
@@ -850,7 +759,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:P495"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
@@ -4053,7 +3962,7 @@
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
@@ -4115,7 +4024,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
@@ -4177,7 +4086,7 @@
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
@@ -4239,7 +4148,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
@@ -4301,7 +4210,7 @@
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
@@ -4363,7 +4272,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
@@ -4425,7 +4334,7 @@
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
@@ -4487,7 +4396,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
@@ -4549,7 +4458,7 @@
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
@@ -4611,7 +4520,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
@@ -4673,7 +4582,7 @@
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
@@ -4735,7 +4644,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
@@ -4797,7 +4706,7 @@
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
@@ -4859,7 +4768,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
@@ -4921,7 +4830,7 @@
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
@@ -4983,7 +4892,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
@@ -5045,7 +4954,7 @@
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
@@ -5107,7 +5016,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
@@ -5169,7 +5078,7 @@
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
@@ -5227,7 +5136,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
@@ -5285,7 +5194,7 @@
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B73" s="2" t="inlineStr">
@@ -5343,7 +5252,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
@@ -5401,7 +5310,7 @@
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B75" s="2" t="inlineStr">
@@ -5459,7 +5368,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
@@ -5517,7 +5426,7 @@
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B77" s="2" t="inlineStr">
@@ -5579,7 +5488,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
@@ -5641,7 +5550,7 @@
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B79" s="2" t="inlineStr">
@@ -5703,7 +5612,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
@@ -5765,7 +5674,7 @@
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B81" s="2" t="inlineStr">
@@ -5827,7 +5736,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
@@ -5889,7 +5798,7 @@
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B83" s="2" t="inlineStr">
@@ -5951,7 +5860,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
@@ -6013,7 +5922,7 @@
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B85" s="2" t="inlineStr">
@@ -6075,7 +5984,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">
@@ -6137,7 +6046,7 @@
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B87" s="2" t="inlineStr">
@@ -6199,7 +6108,7 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B88" s="2" t="inlineStr">
@@ -6261,7 +6170,7 @@
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B89" s="2" t="inlineStr">
@@ -6323,7 +6232,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B90" s="2" t="inlineStr">
@@ -6385,7 +6294,7 @@
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B91" s="2" t="inlineStr">
@@ -6447,7 +6356,7 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B92" s="2" t="inlineStr">
@@ -6509,7 +6418,7 @@
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B93" s="2" t="inlineStr">
@@ -6571,7 +6480,7 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B94" s="2" t="inlineStr">
@@ -6633,7 +6542,7 @@
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B95" s="2" t="inlineStr">
@@ -6691,7 +6600,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B96" s="2" t="inlineStr">
@@ -6749,7 +6658,7 @@
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B97" s="2" t="inlineStr">
@@ -6807,7 +6716,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B98" s="2" t="inlineStr">
@@ -6865,7 +6774,7 @@
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B99" s="2" t="inlineStr">
@@ -6923,7 +6832,7 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B100" s="2" t="inlineStr">
@@ -6981,7 +6890,7 @@
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B101" s="2" t="inlineStr">
@@ -7047,7 +6956,7 @@
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B102" s="2" t="inlineStr">
@@ -7113,7 +7022,7 @@
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B103" s="2" t="inlineStr">
@@ -7179,7 +7088,7 @@
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B104" s="2" t="inlineStr">
@@ -9519,7 +9428,7 @@
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
         <is>
-          <t>220kV Kanakapura</t>
+          <t>220kV Kanakpura</t>
         </is>
       </c>
       <c r="B142" s="2" t="inlineStr">
@@ -9581,7 +9490,7 @@
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
         <is>
-          <t>220kV Kanakapura</t>
+          <t>220kV Kanakpura</t>
         </is>
       </c>
       <c r="B143" s="2" t="inlineStr">
@@ -9643,7 +9552,7 @@
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
         <is>
-          <t>220kV Kanakapura</t>
+          <t>220kV Kanakpura</t>
         </is>
       </c>
       <c r="B144" s="2" t="inlineStr">
@@ -9705,7 +9614,7 @@
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
         <is>
-          <t>220kV Kanakapura</t>
+          <t>220kV Kanakpura</t>
         </is>
       </c>
       <c r="B145" s="2" t="inlineStr">
@@ -9767,7 +9676,7 @@
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
         <is>
-          <t>220kV Kanakapura</t>
+          <t>220kV Kanakpura</t>
         </is>
       </c>
       <c r="B146" s="2" t="inlineStr">
@@ -9829,7 +9738,7 @@
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
         <is>
-          <t>220kV Kanakapura</t>
+          <t>220kV Kanakpura</t>
         </is>
       </c>
       <c r="B147" s="2" t="inlineStr">
@@ -9891,7 +9800,7 @@
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
         <is>
-          <t>220kV Kanakapura</t>
+          <t>220kV Kanakpura</t>
         </is>
       </c>
       <c r="B148" s="2" t="inlineStr">
@@ -9953,7 +9862,7 @@
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
         <is>
-          <t>220kV Kanakapura</t>
+          <t>220kV Kanakpura</t>
         </is>
       </c>
       <c r="B149" s="2" t="inlineStr">
@@ -10015,7 +9924,7 @@
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
         <is>
-          <t>220kV Kanakapura</t>
+          <t>220kV Kanakpura</t>
         </is>
       </c>
       <c r="B150" s="2" t="inlineStr">
@@ -10077,7 +9986,7 @@
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
         <is>
-          <t>220kV Kanakapura</t>
+          <t>220kV Kanakpura</t>
         </is>
       </c>
       <c r="B151" s="2" t="inlineStr">
@@ -10139,7 +10048,7 @@
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
         <is>
-          <t>220kV Kanakapura</t>
+          <t>220kV Kanakpura</t>
         </is>
       </c>
       <c r="B152" s="2" t="inlineStr">
@@ -10201,7 +10110,7 @@
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
         <is>
-          <t>220kV Kanakapura</t>
+          <t>220kV Kanakpura</t>
         </is>
       </c>
       <c r="B153" s="2" t="inlineStr">
@@ -10263,7 +10172,7 @@
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
         <is>
-          <t>220kV Kanakapura</t>
+          <t>220kV Kanakpura</t>
         </is>
       </c>
       <c r="B154" s="2" t="inlineStr">
@@ -10321,7 +10230,7 @@
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
         <is>
-          <t>220kV Kanakapura</t>
+          <t>220kV Kanakpura</t>
         </is>
       </c>
       <c r="B155" s="2" t="inlineStr">
@@ -10379,7 +10288,7 @@
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
         <is>
-          <t>220kV Kanakapura</t>
+          <t>220kV Kanakpura</t>
         </is>
       </c>
       <c r="B156" s="2" t="inlineStr">
@@ -10437,7 +10346,7 @@
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
         <is>
-          <t>220kV Kanakapura</t>
+          <t>220kV Kanakpura</t>
         </is>
       </c>
       <c r="B157" s="2" t="inlineStr">
@@ -10495,7 +10404,7 @@
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
         <is>
-          <t>220kV Kanakapura</t>
+          <t>220kV Kanakpura</t>
         </is>
       </c>
       <c r="B158" s="2" t="inlineStr">
@@ -10553,7 +10462,7 @@
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
         <is>
-          <t>220kV Kanakapura</t>
+          <t>220kV Kanakpura</t>
         </is>
       </c>
       <c r="B159" s="2" t="inlineStr">
@@ -10611,7 +10520,7 @@
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
         <is>
-          <t>220kV Kanakapura</t>
+          <t>220kV Kanakpura</t>
         </is>
       </c>
       <c r="B160" s="2" t="inlineStr">
@@ -10673,7 +10582,7 @@
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
         <is>
-          <t>220kV Kanakapura</t>
+          <t>220kV Kanakpura</t>
         </is>
       </c>
       <c r="B161" s="2" t="inlineStr">
@@ -10735,7 +10644,7 @@
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
         <is>
-          <t>220kV Kanakapura</t>
+          <t>220kV Kanakpura</t>
         </is>
       </c>
       <c r="B162" s="2" t="inlineStr">
@@ -10797,7 +10706,7 @@
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
         <is>
-          <t>220kV Kanakapura</t>
+          <t>220kV Kanakpura</t>
         </is>
       </c>
       <c r="B163" s="2" t="inlineStr">
@@ -10859,7 +10768,7 @@
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
         <is>
-          <t>220kV Kanakapura</t>
+          <t>220kV Kanakpura</t>
         </is>
       </c>
       <c r="B164" s="2" t="inlineStr">
@@ -10921,7 +10830,7 @@
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
         <is>
-          <t>220kV Kanakapura</t>
+          <t>220kV Kanakpura</t>
         </is>
       </c>
       <c r="B165" s="2" t="inlineStr">
@@ -10983,7 +10892,7 @@
     <row r="166">
       <c r="A166" s="2" t="inlineStr">
         <is>
-          <t>220kV Kanakapura</t>
+          <t>220kV Kanakpura</t>
         </is>
       </c>
       <c r="B166" s="2" t="inlineStr">
@@ -11045,7 +10954,7 @@
     <row r="167">
       <c r="A167" s="2" t="inlineStr">
         <is>
-          <t>220kV Kanakapura</t>
+          <t>220kV Kanakpura</t>
         </is>
       </c>
       <c r="B167" s="2" t="inlineStr">
@@ -11107,7 +11016,7 @@
     <row r="168">
       <c r="A168" s="2" t="inlineStr">
         <is>
-          <t>220kV Kanakapura</t>
+          <t>220kV Kanakpura</t>
         </is>
       </c>
       <c r="B168" s="2" t="inlineStr">
@@ -11169,7 +11078,7 @@
     <row r="169">
       <c r="A169" s="2" t="inlineStr">
         <is>
-          <t>220kV Kanakapura</t>
+          <t>220kV Kanakpura</t>
         </is>
       </c>
       <c r="B169" s="2" t="inlineStr">
@@ -11231,7 +11140,7 @@
     <row r="170">
       <c r="A170" s="2" t="inlineStr">
         <is>
-          <t>220kV Kanakapura</t>
+          <t>220kV Kanakpura</t>
         </is>
       </c>
       <c r="B170" s="2" t="inlineStr">
@@ -11293,7 +11202,7 @@
     <row r="171">
       <c r="A171" s="2" t="inlineStr">
         <is>
-          <t>220kV Kanakapura</t>
+          <t>220kV Kanakpura</t>
         </is>
       </c>
       <c r="B171" s="2" t="inlineStr">
@@ -11355,7 +11264,7 @@
     <row r="172">
       <c r="A172" s="2" t="inlineStr">
         <is>
-          <t>220kV Kanakapura</t>
+          <t>220kV Kanakpura</t>
         </is>
       </c>
       <c r="B172" s="2" t="inlineStr">
@@ -11413,7 +11322,7 @@
     <row r="173">
       <c r="A173" s="2" t="inlineStr">
         <is>
-          <t>220kV Kanakapura</t>
+          <t>220kV Kanakpura</t>
         </is>
       </c>
       <c r="B173" s="2" t="inlineStr">
@@ -11471,7 +11380,7 @@
     <row r="174">
       <c r="A174" s="2" t="inlineStr">
         <is>
-          <t>220kV Kanakapura</t>
+          <t>220kV Kanakpura</t>
         </is>
       </c>
       <c r="B174" s="2" t="inlineStr">
@@ -11529,7 +11438,7 @@
     <row r="175">
       <c r="A175" s="2" t="inlineStr">
         <is>
-          <t>220kV Kanakapura</t>
+          <t>220kV Kanakpura</t>
         </is>
       </c>
       <c r="B175" s="2" t="inlineStr">
@@ -11587,7 +11496,7 @@
     <row r="176">
       <c r="A176" s="2" t="inlineStr">
         <is>
-          <t>220kV Kanakapura</t>
+          <t>220kV Kanakpura</t>
         </is>
       </c>
       <c r="B176" s="2" t="inlineStr">
@@ -11645,7 +11554,7 @@
     <row r="177">
       <c r="A177" s="2" t="inlineStr">
         <is>
-          <t>220kV Kanakapura</t>
+          <t>220kV Kanakpura</t>
         </is>
       </c>
       <c r="B177" s="2" t="inlineStr">
@@ -11703,7 +11612,7 @@
     <row r="178">
       <c r="A178" s="2" t="inlineStr">
         <is>
-          <t>220kV Kanakapura</t>
+          <t>220kV Kanakpura</t>
         </is>
       </c>
       <c r="B178" s="2" t="inlineStr">
@@ -11765,7 +11674,7 @@
     <row r="179">
       <c r="A179" s="2" t="inlineStr">
         <is>
-          <t>220kV Kanakapura</t>
+          <t>220kV Kanakpura</t>
         </is>
       </c>
       <c r="B179" s="2" t="inlineStr">
@@ -16545,7 +16454,7 @@
     <row r="257">
       <c r="A257" s="2" t="inlineStr">
         <is>
-          <t>220kV Manyatha Tech Park</t>
+          <t>220kV Manyatha Tech Park GIS Station</t>
         </is>
       </c>
       <c r="B257" s="2" t="inlineStr">
@@ -16607,7 +16516,7 @@
     <row r="258">
       <c r="A258" s="2" t="inlineStr">
         <is>
-          <t>220kV Manyatha Tech Park</t>
+          <t>220kV Manyatha Tech Park GIS Station</t>
         </is>
       </c>
       <c r="B258" s="2" t="inlineStr">
@@ -16669,7 +16578,7 @@
     <row r="259">
       <c r="A259" s="2" t="inlineStr">
         <is>
-          <t>220kV Manyatha Tech Park</t>
+          <t>220kV Manyatha Tech Park GIS Station</t>
         </is>
       </c>
       <c r="B259" s="2" t="inlineStr">
@@ -16731,7 +16640,7 @@
     <row r="260">
       <c r="A260" s="2" t="inlineStr">
         <is>
-          <t>220kV Manyatha Tech Park</t>
+          <t>220kV Manyatha Tech Park GIS Station</t>
         </is>
       </c>
       <c r="B260" s="2" t="inlineStr">
@@ -16793,7 +16702,7 @@
     <row r="261">
       <c r="A261" s="2" t="inlineStr">
         <is>
-          <t>220kV Manyatha Tech Park</t>
+          <t>220kV Manyatha Tech Park GIS Station</t>
         </is>
       </c>
       <c r="B261" s="2" t="inlineStr">
@@ -16855,7 +16764,7 @@
     <row r="262">
       <c r="A262" s="2" t="inlineStr">
         <is>
-          <t>220kV Manyatha Tech Park</t>
+          <t>220kV Manyatha Tech Park GIS Station</t>
         </is>
       </c>
       <c r="B262" s="2" t="inlineStr">
@@ -16917,7 +16826,7 @@
     <row r="263">
       <c r="A263" s="2" t="inlineStr">
         <is>
-          <t>220kV Manyatha Tech Park</t>
+          <t>220kV Manyatha Tech Park GIS Station</t>
         </is>
       </c>
       <c r="B263" s="2" t="inlineStr">
@@ -16979,7 +16888,7 @@
     <row r="264">
       <c r="A264" s="2" t="inlineStr">
         <is>
-          <t>220kV Manyatha Tech Park</t>
+          <t>220kV Manyatha Tech Park GIS Station</t>
         </is>
       </c>
       <c r="B264" s="2" t="inlineStr">
@@ -17041,7 +16950,7 @@
     <row r="265">
       <c r="A265" s="2" t="inlineStr">
         <is>
-          <t>220kV Manyatha Tech Park</t>
+          <t>220kV Manyatha Tech Park GIS Station</t>
         </is>
       </c>
       <c r="B265" s="2" t="inlineStr">
@@ -17103,7 +17012,7 @@
     <row r="266">
       <c r="A266" s="2" t="inlineStr">
         <is>
-          <t>220kV Manyatha Tech Park</t>
+          <t>220kV Manyatha Tech Park GIS Station</t>
         </is>
       </c>
       <c r="B266" s="2" t="inlineStr">
@@ -17165,7 +17074,7 @@
     <row r="267">
       <c r="A267" s="2" t="inlineStr">
         <is>
-          <t>220kV Manyatha Tech Park</t>
+          <t>220kV Manyatha Tech Park GIS Station</t>
         </is>
       </c>
       <c r="B267" s="2" t="inlineStr">
@@ -17227,7 +17136,7 @@
     <row r="268">
       <c r="A268" s="2" t="inlineStr">
         <is>
-          <t>220kV Manyatha Tech Park</t>
+          <t>220kV Manyatha Tech Park GIS Station</t>
         </is>
       </c>
       <c r="B268" s="2" t="inlineStr">
@@ -17289,7 +17198,7 @@
     <row r="269">
       <c r="A269" s="2" t="inlineStr">
         <is>
-          <t>220kV Manyatha Tech Park</t>
+          <t>220kV Manyatha Tech Park GIS Station</t>
         </is>
       </c>
       <c r="B269" s="2" t="inlineStr">
@@ -17351,7 +17260,7 @@
     <row r="270">
       <c r="A270" s="2" t="inlineStr">
         <is>
-          <t>220kV Manyatha Tech Park</t>
+          <t>220kV Manyatha Tech Park GIS Station</t>
         </is>
       </c>
       <c r="B270" s="2" t="inlineStr">
@@ -17413,7 +17322,7 @@
     <row r="271">
       <c r="A271" s="2" t="inlineStr">
         <is>
-          <t>220kV Manyatha Tech Park</t>
+          <t>220kV Manyatha Tech Park GIS Station</t>
         </is>
       </c>
       <c r="B271" s="2" t="inlineStr">
@@ -17475,7 +17384,7 @@
     <row r="272">
       <c r="A272" s="2" t="inlineStr">
         <is>
-          <t>220kV Manyatha Tech Park</t>
+          <t>220kV Manyatha Tech Park GIS Station</t>
         </is>
       </c>
       <c r="B272" s="2" t="inlineStr">
@@ -17537,7 +17446,7 @@
     <row r="273">
       <c r="A273" s="2" t="inlineStr">
         <is>
-          <t>220kV Manyatha Tech Park</t>
+          <t>220kV Manyatha Tech Park GIS Station</t>
         </is>
       </c>
       <c r="B273" s="2" t="inlineStr">
@@ -17599,7 +17508,7 @@
     <row r="274">
       <c r="A274" s="2" t="inlineStr">
         <is>
-          <t>220kV Manyatha Tech Park</t>
+          <t>220kV Manyatha Tech Park GIS Station</t>
         </is>
       </c>
       <c r="B274" s="2" t="inlineStr">
@@ -17661,7 +17570,7 @@
     <row r="275">
       <c r="A275" s="2" t="inlineStr">
         <is>
-          <t>220kV Manyatha Tech Park</t>
+          <t>220kV Manyatha Tech Park GIS Station</t>
         </is>
       </c>
       <c r="B275" s="2" t="inlineStr">
@@ -17723,7 +17632,7 @@
     <row r="276">
       <c r="A276" s="2" t="inlineStr">
         <is>
-          <t>220kV Manyatha Tech Park</t>
+          <t>220kV Manyatha Tech Park GIS Station</t>
         </is>
       </c>
       <c r="B276" s="2" t="inlineStr">
@@ -17785,7 +17694,7 @@
     <row r="277">
       <c r="A277" s="2" t="inlineStr">
         <is>
-          <t>220kV Manyatha Tech Park</t>
+          <t>220kV Manyatha Tech Park GIS Station</t>
         </is>
       </c>
       <c r="B277" s="2" t="inlineStr">
@@ -17847,7 +17756,7 @@
     <row r="278">
       <c r="A278" s="2" t="inlineStr">
         <is>
-          <t>220kV Manyatha Tech Park</t>
+          <t>220kV Manyatha Tech Park GIS Station</t>
         </is>
       </c>
       <c r="B278" s="2" t="inlineStr">
@@ -17909,7 +17818,7 @@
     <row r="279">
       <c r="A279" s="2" t="inlineStr">
         <is>
-          <t>220kV Manyatha Tech Park</t>
+          <t>220kV Manyatha Tech Park GIS Station</t>
         </is>
       </c>
       <c r="B279" s="2" t="inlineStr">
@@ -17971,7 +17880,7 @@
     <row r="280">
       <c r="A280" s="2" t="inlineStr">
         <is>
-          <t>220kV Manyatha Tech Park</t>
+          <t>220kV Manyatha Tech Park GIS Station</t>
         </is>
       </c>
       <c r="B280" s="2" t="inlineStr">
@@ -18033,7 +17942,7 @@
     <row r="281">
       <c r="A281" s="2" t="inlineStr">
         <is>
-          <t>220kV Manyatha Tech Park</t>
+          <t>220kV Manyatha Tech Park GIS Station</t>
         </is>
       </c>
       <c r="B281" s="2" t="inlineStr">
@@ -18095,7 +18004,7 @@
     <row r="282">
       <c r="A282" s="2" t="inlineStr">
         <is>
-          <t>220kV Manyatha Tech Park</t>
+          <t>220kV Manyatha Tech Park GIS Station</t>
         </is>
       </c>
       <c r="B282" s="2" t="inlineStr">
@@ -18157,7 +18066,7 @@
     <row r="283">
       <c r="A283" s="2" t="inlineStr">
         <is>
-          <t>220kV Manyatha Tech Park</t>
+          <t>220kV Manyatha Tech Park GIS Station</t>
         </is>
       </c>
       <c r="B283" s="2" t="inlineStr">
@@ -18219,7 +18128,7 @@
     <row r="284">
       <c r="A284" s="2" t="inlineStr">
         <is>
-          <t>220kV Manyatha Tech Park</t>
+          <t>220kV Manyatha Tech Park GIS Station</t>
         </is>
       </c>
       <c r="B284" s="2" t="inlineStr">
@@ -18281,7 +18190,7 @@
     <row r="285">
       <c r="A285" s="2" t="inlineStr">
         <is>
-          <t>220kV Manyatha Tech Park</t>
+          <t>220kV Manyatha Tech Park GIS Station</t>
         </is>
       </c>
       <c r="B285" s="2" t="inlineStr">
@@ -18343,7 +18252,7 @@
     <row r="286">
       <c r="A286" s="2" t="inlineStr">
         <is>
-          <t>220kV Manyatha Tech Park</t>
+          <t>220kV Manyatha Tech Park GIS Station</t>
         </is>
       </c>
       <c r="B286" s="2" t="inlineStr">
@@ -18405,7 +18314,7 @@
     <row r="287">
       <c r="A287" s="2" t="inlineStr">
         <is>
-          <t>220kV Manyatha Tech Park</t>
+          <t>220kV Manyatha Tech Park GIS Station</t>
         </is>
       </c>
       <c r="B287" s="2" t="inlineStr">
@@ -18467,7 +18376,7 @@
     <row r="288">
       <c r="A288" s="2" t="inlineStr">
         <is>
-          <t>220kV Manyatha Tech Park</t>
+          <t>220kV Manyatha Tech Park GIS Station</t>
         </is>
       </c>
       <c r="B288" s="2" t="inlineStr">
@@ -18529,7 +18438,7 @@
     <row r="289">
       <c r="A289" s="2" t="inlineStr">
         <is>
-          <t>220kV Manyatha Tech Park</t>
+          <t>220kV Manyatha Tech Park GIS Station</t>
         </is>
       </c>
       <c r="B289" s="2" t="inlineStr">
@@ -18591,7 +18500,7 @@
     <row r="290">
       <c r="A290" s="2" t="inlineStr">
         <is>
-          <t>220kV Manyatha Tech Park</t>
+          <t>220kV Manyatha Tech Park GIS Station</t>
         </is>
       </c>
       <c r="B290" s="2" t="inlineStr">
@@ -18653,7 +18562,7 @@
     <row r="291">
       <c r="A291" s="2" t="inlineStr">
         <is>
-          <t>220kV Manyatha Tech Park</t>
+          <t>220kV Manyatha Tech Park GIS Station</t>
         </is>
       </c>
       <c r="B291" s="2" t="inlineStr">
@@ -18715,7 +18624,7 @@
     <row r="292">
       <c r="A292" s="2" t="inlineStr">
         <is>
-          <t>220kV Manyatha Tech Park</t>
+          <t>220kV Manyatha Tech Park GIS Station</t>
         </is>
       </c>
       <c r="B292" s="2" t="inlineStr">
@@ -18777,7 +18686,7 @@
     <row r="293">
       <c r="A293" s="2" t="inlineStr">
         <is>
-          <t>220kV Manyatha Tech Park</t>
+          <t>220kV Manyatha Tech Park GIS Station</t>
         </is>
       </c>
       <c r="B293" s="2" t="inlineStr">
@@ -18839,7 +18748,7 @@
     <row r="294">
       <c r="A294" s="2" t="inlineStr">
         <is>
-          <t>220kV Manyatha Tech Park</t>
+          <t>220kV Manyatha Tech Park GIS Station</t>
         </is>
       </c>
       <c r="B294" s="2" t="inlineStr">
@@ -18901,7 +18810,7 @@
     <row r="295">
       <c r="A295" s="2" t="inlineStr">
         <is>
-          <t>220kV Manyatha Tech Park</t>
+          <t>220kV Manyatha Tech Park GIS Station</t>
         </is>
       </c>
       <c r="B295" s="2" t="inlineStr">
@@ -18963,7 +18872,7 @@
     <row r="296">
       <c r="A296" s="2" t="inlineStr">
         <is>
-          <t>220kV Manyatha Tech Park</t>
+          <t>220kV Manyatha Tech Park GIS Station</t>
         </is>
       </c>
       <c r="B296" s="2" t="inlineStr">
@@ -19025,7 +18934,7 @@
     <row r="297">
       <c r="A297" s="2" t="inlineStr">
         <is>
-          <t>220kV Manyatha Tech Park</t>
+          <t>220kV Manyatha Tech Park GIS Station</t>
         </is>
       </c>
       <c r="B297" s="2" t="inlineStr">
@@ -19087,7 +18996,7 @@
     <row r="298">
       <c r="A298" s="2" t="inlineStr">
         <is>
-          <t>220kV Manyatha Tech Park</t>
+          <t>220kV Manyatha Tech Park GIS Station</t>
         </is>
       </c>
       <c r="B298" s="2" t="inlineStr">
@@ -19149,7 +19058,7 @@
     <row r="299">
       <c r="A299" s="2" t="inlineStr">
         <is>
-          <t>220kV Manyatha Tech Park</t>
+          <t>220kV Manyatha Tech Park GIS Station</t>
         </is>
       </c>
       <c r="B299" s="2" t="inlineStr">
@@ -19215,7 +19124,7 @@
     <row r="300">
       <c r="A300" s="2" t="inlineStr">
         <is>
-          <t>220kV Manyatha Tech Park</t>
+          <t>220kV Manyatha Tech Park GIS Station</t>
         </is>
       </c>
       <c r="B300" s="2" t="inlineStr">
@@ -19281,7 +19190,7 @@
     <row r="301">
       <c r="A301" s="2" t="inlineStr">
         <is>
-          <t>220kV Manyatha Tech Park</t>
+          <t>220kV Manyatha Tech Park GIS Station</t>
         </is>
       </c>
       <c r="B301" s="2" t="inlineStr">
@@ -19347,7 +19256,7 @@
     <row r="302">
       <c r="A302" s="2" t="inlineStr">
         <is>
-          <t>220kV Manyatha Tech Park</t>
+          <t>220kV Manyatha Tech Park GIS Station</t>
         </is>
       </c>
       <c r="B302" s="2" t="inlineStr">
@@ -26623,7 +26532,7 @@
     <row r="420">
       <c r="A420" s="2" t="inlineStr">
         <is>
-          <t>400kV DHP</t>
+          <t>400kV Devanahalli Hardware Park</t>
         </is>
       </c>
       <c r="B420" s="2" t="inlineStr">
@@ -26685,7 +26594,7 @@
     <row r="421">
       <c r="A421" s="2" t="inlineStr">
         <is>
-          <t>400kV DHP</t>
+          <t>400kV Devanahalli Hardware Park</t>
         </is>
       </c>
       <c r="B421" s="2" t="inlineStr">
@@ -26747,7 +26656,7 @@
     <row r="422">
       <c r="A422" s="2" t="inlineStr">
         <is>
-          <t>400kV DHP</t>
+          <t>400kV Devanahalli Hardware Park</t>
         </is>
       </c>
       <c r="B422" s="2" t="inlineStr">
@@ -26809,7 +26718,7 @@
     <row r="423">
       <c r="A423" s="2" t="inlineStr">
         <is>
-          <t>400kV DHP</t>
+          <t>400kV Devanahalli Hardware Park</t>
         </is>
       </c>
       <c r="B423" s="2" t="inlineStr">
@@ -26867,7 +26776,7 @@
     <row r="424">
       <c r="A424" s="2" t="inlineStr">
         <is>
-          <t>400kV DHP</t>
+          <t>400kV Devanahalli Hardware Park</t>
         </is>
       </c>
       <c r="B424" s="2" t="inlineStr">
@@ -26925,7 +26834,7 @@
     <row r="425">
       <c r="A425" s="2" t="inlineStr">
         <is>
-          <t>400kV DHP</t>
+          <t>400kV Devanahalli Hardware Park</t>
         </is>
       </c>
       <c r="B425" s="2" t="inlineStr">
@@ -26983,7 +26892,7 @@
     <row r="426">
       <c r="A426" s="2" t="inlineStr">
         <is>
-          <t>400kV DHP</t>
+          <t>400kV Devanahalli Hardware Park</t>
         </is>
       </c>
       <c r="B426" s="2" t="inlineStr">
@@ -27045,7 +26954,7 @@
     <row r="427">
       <c r="A427" s="2" t="inlineStr">
         <is>
-          <t>400kV DHP</t>
+          <t>400kV Devanahalli Hardware Park</t>
         </is>
       </c>
       <c r="B427" s="2" t="inlineStr">
@@ -27107,7 +27016,7 @@
     <row r="428">
       <c r="A428" s="2" t="inlineStr">
         <is>
-          <t>400kV DHP</t>
+          <t>400kV Devanahalli Hardware Park</t>
         </is>
       </c>
       <c r="B428" s="2" t="inlineStr">
@@ -27169,7 +27078,7 @@
     <row r="429">
       <c r="A429" s="2" t="inlineStr">
         <is>
-          <t>400kV DHP</t>
+          <t>400kV Devanahalli Hardware Park</t>
         </is>
       </c>
       <c r="B429" s="2" t="inlineStr">
@@ -27231,7 +27140,7 @@
     <row r="430">
       <c r="A430" s="2" t="inlineStr">
         <is>
-          <t>400kV DHP</t>
+          <t>400kV Devanahalli Hardware Park</t>
         </is>
       </c>
       <c r="B430" s="2" t="inlineStr">
@@ -27293,7 +27202,7 @@
     <row r="431">
       <c r="A431" s="2" t="inlineStr">
         <is>
-          <t>400kV DHP</t>
+          <t>400kV Devanahalli Hardware Park</t>
         </is>
       </c>
       <c r="B431" s="2" t="inlineStr">
@@ -27355,7 +27264,7 @@
     <row r="432">
       <c r="A432" s="2" t="inlineStr">
         <is>
-          <t>400kV DHP</t>
+          <t>400kV Devanahalli Hardware Park</t>
         </is>
       </c>
       <c r="B432" s="2" t="inlineStr">
@@ -27417,7 +27326,7 @@
     <row r="433">
       <c r="A433" s="2" t="inlineStr">
         <is>
-          <t>400kV DHP</t>
+          <t>400kV Devanahalli Hardware Park</t>
         </is>
       </c>
       <c r="B433" s="2" t="inlineStr">
@@ -27479,7 +27388,7 @@
     <row r="434">
       <c r="A434" s="2" t="inlineStr">
         <is>
-          <t>400kV DHP</t>
+          <t>400kV Devanahalli Hardware Park</t>
         </is>
       </c>
       <c r="B434" s="2" t="inlineStr">
@@ -27541,7 +27450,7 @@
     <row r="435">
       <c r="A435" s="2" t="inlineStr">
         <is>
-          <t>400kV DHP</t>
+          <t>400kV Devanahalli Hardware Park</t>
         </is>
       </c>
       <c r="B435" s="2" t="inlineStr">
@@ -27603,7 +27512,7 @@
     <row r="436">
       <c r="A436" s="2" t="inlineStr">
         <is>
-          <t>400kV DHP</t>
+          <t>400kV Devanahalli Hardware Park</t>
         </is>
       </c>
       <c r="B436" s="2" t="inlineStr">
@@ -27665,7 +27574,7 @@
     <row r="437">
       <c r="A437" s="2" t="inlineStr">
         <is>
-          <t>400kV DHP</t>
+          <t>400kV Devanahalli Hardware Park</t>
         </is>
       </c>
       <c r="B437" s="2" t="inlineStr">
@@ -27727,7 +27636,7 @@
     <row r="438">
       <c r="A438" s="2" t="inlineStr">
         <is>
-          <t>400kV DHP</t>
+          <t>400kV Devanahalli Hardware Park</t>
         </is>
       </c>
       <c r="B438" s="2" t="inlineStr">
@@ -27789,7 +27698,7 @@
     <row r="439">
       <c r="A439" s="2" t="inlineStr">
         <is>
-          <t>400kV DHP</t>
+          <t>400kV Devanahalli Hardware Park</t>
         </is>
       </c>
       <c r="B439" s="2" t="inlineStr">
@@ -27851,7 +27760,7 @@
     <row r="440">
       <c r="A440" s="2" t="inlineStr">
         <is>
-          <t>400kV DHP</t>
+          <t>400kV Devanahalli Hardware Park</t>
         </is>
       </c>
       <c r="B440" s="2" t="inlineStr">
@@ -27913,7 +27822,7 @@
     <row r="441">
       <c r="A441" s="2" t="inlineStr">
         <is>
-          <t>400kV DHP</t>
+          <t>400kV Devanahalli Hardware Park</t>
         </is>
       </c>
       <c r="B441" s="2" t="inlineStr">
@@ -27975,7 +27884,7 @@
     <row r="442">
       <c r="A442" s="2" t="inlineStr">
         <is>
-          <t>400kV DHP</t>
+          <t>400kV Devanahalli Hardware Park</t>
         </is>
       </c>
       <c r="B442" s="2" t="inlineStr">
@@ -28037,7 +27946,7 @@
     <row r="443">
       <c r="A443" s="2" t="inlineStr">
         <is>
-          <t>400kV DHP</t>
+          <t>400kV Devanahalli Hardware Park</t>
         </is>
       </c>
       <c r="B443" s="2" t="inlineStr">
@@ -28099,7 +28008,7 @@
     <row r="444">
       <c r="A444" s="2" t="inlineStr">
         <is>
-          <t>400kV DHP</t>
+          <t>400kV Devanahalli Hardware Park</t>
         </is>
       </c>
       <c r="B444" s="2" t="inlineStr">
@@ -28161,7 +28070,7 @@
     <row r="445">
       <c r="A445" s="2" t="inlineStr">
         <is>
-          <t>400kV DHP</t>
+          <t>400kV Devanahalli Hardware Park</t>
         </is>
       </c>
       <c r="B445" s="2" t="inlineStr">
@@ -28223,7 +28132,7 @@
     <row r="446">
       <c r="A446" s="2" t="inlineStr">
         <is>
-          <t>400kV DHP</t>
+          <t>400kV Devanahalli Hardware Park</t>
         </is>
       </c>
       <c r="B446" s="2" t="inlineStr">
@@ -28285,7 +28194,7 @@
     <row r="447">
       <c r="A447" s="2" t="inlineStr">
         <is>
-          <t>400kV DHP</t>
+          <t>400kV Devanahalli Hardware Park</t>
         </is>
       </c>
       <c r="B447" s="2" t="inlineStr">
@@ -28347,7 +28256,7 @@
     <row r="448">
       <c r="A448" s="2" t="inlineStr">
         <is>
-          <t>400kV DHP</t>
+          <t>400kV Devanahalli Hardware Park</t>
         </is>
       </c>
       <c r="B448" s="2" t="inlineStr">
@@ -28409,7 +28318,7 @@
     <row r="449">
       <c r="A449" s="2" t="inlineStr">
         <is>
-          <t>400kV DHP</t>
+          <t>400kV Devanahalli Hardware Park</t>
         </is>
       </c>
       <c r="B449" s="2" t="inlineStr">
@@ -28471,7 +28380,7 @@
     <row r="450">
       <c r="A450" s="2" t="inlineStr">
         <is>
-          <t>400kV DHP</t>
+          <t>400kV Devanahalli Hardware Park</t>
         </is>
       </c>
       <c r="B450" s="2" t="inlineStr">
@@ -28533,7 +28442,7 @@
     <row r="451">
       <c r="A451" s="2" t="inlineStr">
         <is>
-          <t>400kV DHP</t>
+          <t>400kV Devanahalli Hardware Park</t>
         </is>
       </c>
       <c r="B451" s="2" t="inlineStr">
@@ -28595,7 +28504,7 @@
     <row r="452">
       <c r="A452" s="2" t="inlineStr">
         <is>
-          <t>400kV DHP</t>
+          <t>400kV Devanahalli Hardware Park</t>
         </is>
       </c>
       <c r="B452" s="2" t="inlineStr">
@@ -28657,7 +28566,7 @@
     <row r="453">
       <c r="A453" s="2" t="inlineStr">
         <is>
-          <t>400kV DHP</t>
+          <t>400kV Devanahalli Hardware Park</t>
         </is>
       </c>
       <c r="B453" s="2" t="inlineStr">
@@ -28715,7 +28624,7 @@
     <row r="454">
       <c r="A454" s="2" t="inlineStr">
         <is>
-          <t>400kV DHP</t>
+          <t>400kV Devanahalli Hardware Park</t>
         </is>
       </c>
       <c r="B454" s="2" t="inlineStr">
@@ -28773,7 +28682,7 @@
     <row r="455">
       <c r="A455" s="2" t="inlineStr">
         <is>
-          <t>400kV DHP</t>
+          <t>400kV Devanahalli Hardware Park</t>
         </is>
       </c>
       <c r="B455" s="2" t="inlineStr">
@@ -28831,7 +28740,7 @@
     <row r="456">
       <c r="A456" s="2" t="inlineStr">
         <is>
-          <t>400kV DHP</t>
+          <t>400kV Devanahalli Hardware Park</t>
         </is>
       </c>
       <c r="B456" s="2" t="inlineStr">
@@ -28889,7 +28798,7 @@
     <row r="457">
       <c r="A457" s="2" t="inlineStr">
         <is>
-          <t>400kV DHP</t>
+          <t>400kV Devanahalli Hardware Park</t>
         </is>
       </c>
       <c r="B457" s="2" t="inlineStr">
@@ -28947,7 +28856,7 @@
     <row r="458">
       <c r="A458" s="2" t="inlineStr">
         <is>
-          <t>400kV DHP</t>
+          <t>400kV Devanahalli Hardware Park</t>
         </is>
       </c>
       <c r="B458" s="2" t="inlineStr">
@@ -29005,7 +28914,7 @@
     <row r="459">
       <c r="A459" s="2" t="inlineStr">
         <is>
-          <t>400kV DHP</t>
+          <t>400kV Devanahalli Hardware Park</t>
         </is>
       </c>
       <c r="B459" s="2" t="inlineStr">
@@ -29059,7 +28968,7 @@
     <row r="460">
       <c r="A460" s="2" t="inlineStr">
         <is>
-          <t>400kV DHP</t>
+          <t>400kV Devanahalli Hardware Park</t>
         </is>
       </c>
       <c r="B460" s="2" t="inlineStr">

</xml_diff>

<commit_message>
fix(seed): correct station name mismatches and add missing 400kV DHP to mapping
- equipment_seed.xlsx Equipment sheet: rename 3 stations to match KPTCL mapping
    220kV EDC -> 220kV Sir M V EDC GIS
    220kV Kanakapura -> 66kV Kanakapura
    220kV Manyatha Tech Park -> 220kV Manyatha Tech Park GIS Station
- equipment_seed.xlsx Departments sheet: rewrite hierarchy with correct
  Bangalore Zone circle/division names (BRAZ, BMAZ North, BMAZ South, Ramanagara)
  replacing the stale Bengaluru Transmission Circle naming
- KPTCL_Substation_Mapping.xlsx: add 400kV DHP under Bangalore Zone / BMAZ South / Hoody

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/equipment_seed.xlsx
+++ b/equipment_seed.xlsx
@@ -447,17 +447,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Bengaluru Zone</t>
+          <t>Bangalore Zone</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Bengaluru Transmission Circle</t>
+          <t>BRAZ</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>RT North Division</t>
+          <t>Begur</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -469,39 +469,39 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Bengaluru Zone</t>
+          <t>Bangalore Zone</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Bengaluru Transmission Circle</t>
+          <t>BMAZ South</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>RT East Division</t>
+          <t>Hoody</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Bengaluru Zone</t>
+          <t>Bangalore Zone</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Bengaluru Transmission Circle</t>
+          <t>Ramanagara</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>RT East Division</t>
+          <t>Yerandanahally</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -513,39 +513,39 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Bengaluru Zone</t>
+          <t>Bangalore Zone</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Bengaluru Transmission Circle</t>
+          <t>Ramanagara</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>RT South Division</t>
+          <t>Kanakapura</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>220kV Kanakapura</t>
+          <t>66kV Kanakapura</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Bengaluru Zone</t>
+          <t>Bangalore Zone</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Kolar Transmission Circle</t>
+          <t>BRAZ</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Kolar Division</t>
+          <t>Kolar</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -557,17 +557,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Bengaluru Zone</t>
+          <t>Bangalore Zone</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Kolar Transmission Circle</t>
+          <t>BRAZ</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Kolar Division</t>
+          <t>Malur</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -579,39 +579,39 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Bengaluru Zone</t>
+          <t>Bangalore Zone</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Bengaluru Transmission Circle</t>
+          <t>BMAZ North</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>RT North Division</t>
+          <t>Hebbal</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>220kV Manyatha Tech Park</t>
+          <t>220kV Manyatha Tech Park GIS Station</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Bengaluru Zone</t>
+          <t>Bangalore Zone</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Bengaluru Transmission Circle</t>
+          <t>BMAZ North</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>RT South Division</t>
+          <t>NRS</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -623,17 +623,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Bengaluru Zone</t>
+          <t>Bangalore Zone</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Bengaluru Transmission Circle</t>
+          <t>Ramanagara</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>RT East Division</t>
+          <t>Yerandanahally</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -645,17 +645,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Bengaluru Zone</t>
+          <t>Bangalore Zone</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Bengaluru Transmission Circle</t>
+          <t>BMAZ South</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>RT East Division</t>
+          <t>Hoody</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -667,17 +667,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Bengaluru Zone</t>
+          <t>Bangalore Zone</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Bengaluru Transmission Circle</t>
+          <t>BMAZ South</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>RT East Division</t>
+          <t>Hoody</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -3674,7 +3674,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -3731,7 +3731,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -3788,7 +3788,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -3845,7 +3845,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -3902,7 +3902,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -3959,7 +3959,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -4016,7 +4016,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -4073,7 +4073,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -4130,7 +4130,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -4187,7 +4187,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -4244,7 +4244,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -4301,7 +4301,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -4358,7 +4358,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -4415,7 +4415,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -4472,7 +4472,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -4529,7 +4529,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -4586,7 +4586,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -4643,7 +4643,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -4700,7 +4700,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -4752,7 +4752,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -4804,7 +4804,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -4856,7 +4856,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -4908,7 +4908,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -4960,7 +4960,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -5012,7 +5012,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -5069,7 +5069,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -5126,7 +5126,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -5183,7 +5183,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -5240,7 +5240,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -5297,7 +5297,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -5354,7 +5354,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -5411,7 +5411,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -5468,7 +5468,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -5525,7 +5525,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -5582,7 +5582,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -5639,7 +5639,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -5696,7 +5696,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -5753,7 +5753,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -5810,7 +5810,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -5867,7 +5867,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -5924,7 +5924,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -5981,7 +5981,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -6038,7 +6038,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -6090,7 +6090,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -6142,7 +6142,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -6194,7 +6194,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -6246,7 +6246,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -6298,7 +6298,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -6350,7 +6350,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -6412,7 +6412,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -6474,7 +6474,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -6536,7 +6536,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>220kV EDC</t>
+          <t>220kV Sir M V EDC GIS</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -8682,7 +8682,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>220kV Kanakapura</t>
+          <t>66kV Kanakapura</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -8739,7 +8739,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>220kV Kanakapura</t>
+          <t>66kV Kanakapura</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
@@ -8796,7 +8796,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>220kV Kanakapura</t>
+          <t>66kV Kanakapura</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
@@ -8853,7 +8853,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>220kV Kanakapura</t>
+          <t>66kV Kanakapura</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
@@ -8910,7 +8910,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>220kV Kanakapura</t>
+          <t>66kV Kanakapura</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
@@ -8967,7 +8967,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>220kV Kanakapura</t>
+          <t>66kV Kanakapura</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
@@ -9024,7 +9024,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>220kV Kanakapura</t>
+          <t>66kV Kanakapura</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
@@ -9081,7 +9081,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>220kV Kanakapura</t>
+          <t>66kV Kanakapura</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
@@ -9138,7 +9138,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>220kV Kanakapura</t>
+          <t>66kV Kanakapura</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
@@ -9195,7 +9195,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>220kV Kanakapura</t>
+          <t>66kV Kanakapura</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -9252,7 +9252,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>220kV Kanakapura</t>
+          <t>66kV Kanakapura</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -9309,7 +9309,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>220kV Kanakapura</t>
+          <t>66kV Kanakapura</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
@@ -9366,7 +9366,7 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>220kV Kanakapura</t>
+          <t>66kV Kanakapura</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
@@ -9418,7 +9418,7 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>220kV Kanakapura</t>
+          <t>66kV Kanakapura</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
@@ -9470,7 +9470,7 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>220kV Kanakapura</t>
+          <t>66kV Kanakapura</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
@@ -9522,7 +9522,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>220kV Kanakapura</t>
+          <t>66kV Kanakapura</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
@@ -9574,7 +9574,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>220kV Kanakapura</t>
+          <t>66kV Kanakapura</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
@@ -9626,7 +9626,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>220kV Kanakapura</t>
+          <t>66kV Kanakapura</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
@@ -9678,7 +9678,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>220kV Kanakapura</t>
+          <t>66kV Kanakapura</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
@@ -9735,7 +9735,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>220kV Kanakapura</t>
+          <t>66kV Kanakapura</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
@@ -9792,7 +9792,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>220kV Kanakapura</t>
+          <t>66kV Kanakapura</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
@@ -9849,7 +9849,7 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>220kV Kanakapura</t>
+          <t>66kV Kanakapura</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
@@ -9906,7 +9906,7 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>220kV Kanakapura</t>
+          <t>66kV Kanakapura</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
@@ -9963,7 +9963,7 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>220kV Kanakapura</t>
+          <t>66kV Kanakapura</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
@@ -10020,7 +10020,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>220kV Kanakapura</t>
+          <t>66kV Kanakapura</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
@@ -10077,7 +10077,7 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>220kV Kanakapura</t>
+          <t>66kV Kanakapura</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
@@ -10134,7 +10134,7 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>220kV Kanakapura</t>
+          <t>66kV Kanakapura</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
@@ -10191,7 +10191,7 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>220kV Kanakapura</t>
+          <t>66kV Kanakapura</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
@@ -10248,7 +10248,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>220kV Kanakapura</t>
+          <t>66kV Kanakapura</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
@@ -10305,7 +10305,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>220kV Kanakapura</t>
+          <t>66kV Kanakapura</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
@@ -10362,7 +10362,7 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>220kV Kanakapura</t>
+          <t>66kV Kanakapura</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
@@ -10414,7 +10414,7 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>220kV Kanakapura</t>
+          <t>66kV Kanakapura</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
@@ -10466,7 +10466,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>220kV Kanakapura</t>
+          <t>66kV Kanakapura</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
@@ -10518,7 +10518,7 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>220kV Kanakapura</t>
+          <t>66kV Kanakapura</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
@@ -10570,7 +10570,7 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>220kV Kanakapura</t>
+          <t>66kV Kanakapura</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
@@ -10622,7 +10622,7 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>220kV Kanakapura</t>
+          <t>66kV Kanakapura</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
@@ -10674,7 +10674,7 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>220kV Kanakapura</t>
+          <t>66kV Kanakapura</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
@@ -10731,7 +10731,7 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>220kV Kanakapura</t>
+          <t>66kV Kanakapura</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
@@ -15107,7 +15107,7 @@
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>220kV Manyatha Tech Park</t>
+          <t>220kV Manyatha Tech Park GIS Station</t>
         </is>
       </c>
       <c r="B258" t="inlineStr">
@@ -15164,7 +15164,7 @@
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>220kV Manyatha Tech Park</t>
+          <t>220kV Manyatha Tech Park GIS Station</t>
         </is>
       </c>
       <c r="B259" t="inlineStr">
@@ -15221,7 +15221,7 @@
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>220kV Manyatha Tech Park</t>
+          <t>220kV Manyatha Tech Park GIS Station</t>
         </is>
       </c>
       <c r="B260" t="inlineStr">
@@ -15278,7 +15278,7 @@
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>220kV Manyatha Tech Park</t>
+          <t>220kV Manyatha Tech Park GIS Station</t>
         </is>
       </c>
       <c r="B261" t="inlineStr">
@@ -15335,7 +15335,7 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>220kV Manyatha Tech Park</t>
+          <t>220kV Manyatha Tech Park GIS Station</t>
         </is>
       </c>
       <c r="B262" t="inlineStr">
@@ -15392,7 +15392,7 @@
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>220kV Manyatha Tech Park</t>
+          <t>220kV Manyatha Tech Park GIS Station</t>
         </is>
       </c>
       <c r="B263" t="inlineStr">
@@ -15449,7 +15449,7 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>220kV Manyatha Tech Park</t>
+          <t>220kV Manyatha Tech Park GIS Station</t>
         </is>
       </c>
       <c r="B264" t="inlineStr">
@@ -15506,7 +15506,7 @@
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>220kV Manyatha Tech Park</t>
+          <t>220kV Manyatha Tech Park GIS Station</t>
         </is>
       </c>
       <c r="B265" t="inlineStr">
@@ -15563,7 +15563,7 @@
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>220kV Manyatha Tech Park</t>
+          <t>220kV Manyatha Tech Park GIS Station</t>
         </is>
       </c>
       <c r="B266" t="inlineStr">
@@ -15620,7 +15620,7 @@
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>220kV Manyatha Tech Park</t>
+          <t>220kV Manyatha Tech Park GIS Station</t>
         </is>
       </c>
       <c r="B267" t="inlineStr">
@@ -15677,7 +15677,7 @@
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>220kV Manyatha Tech Park</t>
+          <t>220kV Manyatha Tech Park GIS Station</t>
         </is>
       </c>
       <c r="B268" t="inlineStr">
@@ -15734,7 +15734,7 @@
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>220kV Manyatha Tech Park</t>
+          <t>220kV Manyatha Tech Park GIS Station</t>
         </is>
       </c>
       <c r="B269" t="inlineStr">
@@ -15791,7 +15791,7 @@
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>220kV Manyatha Tech Park</t>
+          <t>220kV Manyatha Tech Park GIS Station</t>
         </is>
       </c>
       <c r="B270" t="inlineStr">
@@ -15848,7 +15848,7 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>220kV Manyatha Tech Park</t>
+          <t>220kV Manyatha Tech Park GIS Station</t>
         </is>
       </c>
       <c r="B271" t="inlineStr">
@@ -15905,7 +15905,7 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>220kV Manyatha Tech Park</t>
+          <t>220kV Manyatha Tech Park GIS Station</t>
         </is>
       </c>
       <c r="B272" t="inlineStr">
@@ -15962,7 +15962,7 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>220kV Manyatha Tech Park</t>
+          <t>220kV Manyatha Tech Park GIS Station</t>
         </is>
       </c>
       <c r="B273" t="inlineStr">
@@ -16019,7 +16019,7 @@
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>220kV Manyatha Tech Park</t>
+          <t>220kV Manyatha Tech Park GIS Station</t>
         </is>
       </c>
       <c r="B274" t="inlineStr">
@@ -16076,7 +16076,7 @@
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>220kV Manyatha Tech Park</t>
+          <t>220kV Manyatha Tech Park GIS Station</t>
         </is>
       </c>
       <c r="B275" t="inlineStr">
@@ -16133,7 +16133,7 @@
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>220kV Manyatha Tech Park</t>
+          <t>220kV Manyatha Tech Park GIS Station</t>
         </is>
       </c>
       <c r="B276" t="inlineStr">
@@ -16190,7 +16190,7 @@
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>220kV Manyatha Tech Park</t>
+          <t>220kV Manyatha Tech Park GIS Station</t>
         </is>
       </c>
       <c r="B277" t="inlineStr">
@@ -16247,7 +16247,7 @@
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>220kV Manyatha Tech Park</t>
+          <t>220kV Manyatha Tech Park GIS Station</t>
         </is>
       </c>
       <c r="B278" t="inlineStr">
@@ -16304,7 +16304,7 @@
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>220kV Manyatha Tech Park</t>
+          <t>220kV Manyatha Tech Park GIS Station</t>
         </is>
       </c>
       <c r="B279" t="inlineStr">
@@ -16361,7 +16361,7 @@
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>220kV Manyatha Tech Park</t>
+          <t>220kV Manyatha Tech Park GIS Station</t>
         </is>
       </c>
       <c r="B280" t="inlineStr">
@@ -16418,7 +16418,7 @@
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>220kV Manyatha Tech Park</t>
+          <t>220kV Manyatha Tech Park GIS Station</t>
         </is>
       </c>
       <c r="B281" t="inlineStr">
@@ -16475,7 +16475,7 @@
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>220kV Manyatha Tech Park</t>
+          <t>220kV Manyatha Tech Park GIS Station</t>
         </is>
       </c>
       <c r="B282" t="inlineStr">
@@ -16532,7 +16532,7 @@
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>220kV Manyatha Tech Park</t>
+          <t>220kV Manyatha Tech Park GIS Station</t>
         </is>
       </c>
       <c r="B283" t="inlineStr">
@@ -16589,7 +16589,7 @@
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>220kV Manyatha Tech Park</t>
+          <t>220kV Manyatha Tech Park GIS Station</t>
         </is>
       </c>
       <c r="B284" t="inlineStr">
@@ -16646,7 +16646,7 @@
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>220kV Manyatha Tech Park</t>
+          <t>220kV Manyatha Tech Park GIS Station</t>
         </is>
       </c>
       <c r="B285" t="inlineStr">
@@ -16703,7 +16703,7 @@
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>220kV Manyatha Tech Park</t>
+          <t>220kV Manyatha Tech Park GIS Station</t>
         </is>
       </c>
       <c r="B286" t="inlineStr">
@@ -16760,7 +16760,7 @@
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>220kV Manyatha Tech Park</t>
+          <t>220kV Manyatha Tech Park GIS Station</t>
         </is>
       </c>
       <c r="B287" t="inlineStr">
@@ -16817,7 +16817,7 @@
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>220kV Manyatha Tech Park</t>
+          <t>220kV Manyatha Tech Park GIS Station</t>
         </is>
       </c>
       <c r="B288" t="inlineStr">
@@ -16874,7 +16874,7 @@
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>220kV Manyatha Tech Park</t>
+          <t>220kV Manyatha Tech Park GIS Station</t>
         </is>
       </c>
       <c r="B289" t="inlineStr">
@@ -16931,7 +16931,7 @@
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>220kV Manyatha Tech Park</t>
+          <t>220kV Manyatha Tech Park GIS Station</t>
         </is>
       </c>
       <c r="B290" t="inlineStr">
@@ -16988,7 +16988,7 @@
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t>220kV Manyatha Tech Park</t>
+          <t>220kV Manyatha Tech Park GIS Station</t>
         </is>
       </c>
       <c r="B291" t="inlineStr">
@@ -17045,7 +17045,7 @@
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>220kV Manyatha Tech Park</t>
+          <t>220kV Manyatha Tech Park GIS Station</t>
         </is>
       </c>
       <c r="B292" t="inlineStr">
@@ -17102,7 +17102,7 @@
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>220kV Manyatha Tech Park</t>
+          <t>220kV Manyatha Tech Park GIS Station</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
@@ -17159,7 +17159,7 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>220kV Manyatha Tech Park</t>
+          <t>220kV Manyatha Tech Park GIS Station</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
@@ -17216,7 +17216,7 @@
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>220kV Manyatha Tech Park</t>
+          <t>220kV Manyatha Tech Park GIS Station</t>
         </is>
       </c>
       <c r="B295" t="inlineStr">
@@ -17273,7 +17273,7 @@
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>220kV Manyatha Tech Park</t>
+          <t>220kV Manyatha Tech Park GIS Station</t>
         </is>
       </c>
       <c r="B296" t="inlineStr">
@@ -17330,7 +17330,7 @@
     <row r="297">
       <c r="A297" t="inlineStr">
         <is>
-          <t>220kV Manyatha Tech Park</t>
+          <t>220kV Manyatha Tech Park GIS Station</t>
         </is>
       </c>
       <c r="B297" t="inlineStr">
@@ -17387,7 +17387,7 @@
     <row r="298">
       <c r="A298" t="inlineStr">
         <is>
-          <t>220kV Manyatha Tech Park</t>
+          <t>220kV Manyatha Tech Park GIS Station</t>
         </is>
       </c>
       <c r="B298" t="inlineStr">
@@ -17444,7 +17444,7 @@
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
-          <t>220kV Manyatha Tech Park</t>
+          <t>220kV Manyatha Tech Park GIS Station</t>
         </is>
       </c>
       <c r="B299" t="inlineStr">
@@ -17501,7 +17501,7 @@
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
-          <t>220kV Manyatha Tech Park</t>
+          <t>220kV Manyatha Tech Park GIS Station</t>
         </is>
       </c>
       <c r="B300" t="inlineStr">
@@ -17563,7 +17563,7 @@
     <row r="301">
       <c r="A301" t="inlineStr">
         <is>
-          <t>220kV Manyatha Tech Park</t>
+          <t>220kV Manyatha Tech Park GIS Station</t>
         </is>
       </c>
       <c r="B301" t="inlineStr">
@@ -17625,7 +17625,7 @@
     <row r="302">
       <c r="A302" t="inlineStr">
         <is>
-          <t>220kV Manyatha Tech Park</t>
+          <t>220kV Manyatha Tech Park GIS Station</t>
         </is>
       </c>
       <c r="B302" t="inlineStr">
@@ -17687,7 +17687,7 @@
     <row r="303">
       <c r="A303" t="inlineStr">
         <is>
-          <t>220kV Manyatha Tech Park</t>
+          <t>220kV Manyatha Tech Park GIS Station</t>
         </is>
       </c>
       <c r="B303" t="inlineStr">

</xml_diff>